<commit_message>
Update figure scripts and add new panels for 04_Figures_v1
</commit_message>
<xml_diff>
--- a/04_Figures_v1/F5/c_data/Figure_5_data.xlsx
+++ b/04_Figures_v1/F5/c_data/Figure_5_data.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3017" uniqueCount="3017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3027" uniqueCount="3027">
   <si>
     <t xml:space="preserve">unmerged_color</t>
   </si>
@@ -8997,7 +8997,37 @@
     <t xml:space="preserve">preservation</t>
   </si>
   <si>
+    <t xml:space="preserve">bio_label</t>
+  </si>
+  <si>
     <t xml:space="preserve">Strong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magenta (Magenta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ubiquitin-Proteasome (Yellow)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protein Modification (Turquoise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immune/Complement (Pink)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Translation Machinery (Black)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catabolic Metabolism (Blue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cytoskeletal Remodeling (Brown)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muscle Structure (Green)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red (Red)</t>
   </si>
   <si>
     <t xml:space="preserve">sheet</t>
@@ -76382,185 +76412,215 @@
       <c r="F1" t="s">
         <v>2991</v>
       </c>
+      <c r="G1" t="s">
+        <v>2992</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>19.4888845470859</v>
+        <v>10.6322045154526</v>
       </c>
       <c r="C2" t="n">
-        <v>33.8504120090264</v>
+        <v>14.8902175928694</v>
       </c>
       <c r="D2" t="n">
-        <v>5.12735708514541</v>
+        <v>6.37419143803588</v>
       </c>
       <c r="E2" t="n">
-        <v>139</v>
+        <v>66</v>
       </c>
       <c r="F2" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2994</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" t="n">
-        <v>23.0700843051989</v>
+        <v>17.1724986115383</v>
       </c>
       <c r="C3" t="n">
-        <v>30.6016488916127</v>
+        <v>24.4554446207501</v>
       </c>
       <c r="D3" t="n">
-        <v>15.5385197187852</v>
+        <v>9.88955260232654</v>
       </c>
       <c r="E3" t="n">
-        <v>295</v>
+        <v>225</v>
       </c>
       <c r="F3" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G3" t="s">
+        <v>2995</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>24.6955774310399</v>
+        <v>19.3865194734346</v>
       </c>
       <c r="C4" t="n">
-        <v>35.7149677081741</v>
+        <v>23.7636228049237</v>
       </c>
       <c r="D4" t="n">
-        <v>13.6761871539057</v>
+        <v>15.0094161419456</v>
       </c>
       <c r="E4" t="n">
-        <v>266</v>
+        <v>332</v>
       </c>
       <c r="F4" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G4" t="s">
+        <v>2996</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="n">
-        <v>24.8047047065459</v>
+        <v>19.4551264424704</v>
       </c>
       <c r="C5" t="n">
-        <v>34.1922037910341</v>
+        <v>29.8745177030698</v>
       </c>
       <c r="D5" t="n">
-        <v>15.4172056220576</v>
+        <v>9.03573518187091</v>
       </c>
       <c r="E5" t="n">
-        <v>175</v>
+        <v>94</v>
       </c>
       <c r="F5" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G5" t="s">
+        <v>2997</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>10.6322045154526</v>
+        <v>19.4888845470859</v>
       </c>
       <c r="C6" t="n">
-        <v>14.8902175928694</v>
+        <v>33.8504120090264</v>
       </c>
       <c r="D6" t="n">
-        <v>6.37419143803588</v>
+        <v>5.12735708514541</v>
       </c>
       <c r="E6" t="n">
-        <v>66</v>
+        <v>139</v>
       </c>
       <c r="F6" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G6" t="s">
+        <v>2998</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>19.4551264424704</v>
+        <v>23.0700843051989</v>
       </c>
       <c r="C7" t="n">
-        <v>29.8745177030698</v>
+        <v>30.6016488916127</v>
       </c>
       <c r="D7" t="n">
-        <v>9.03573518187091</v>
+        <v>15.5385197187852</v>
       </c>
       <c r="E7" t="n">
-        <v>94</v>
+        <v>295</v>
       </c>
       <c r="F7" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G7" t="s">
+        <v>2999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" t="n">
-        <v>36.3979475266971</v>
+        <v>24.6955774310399</v>
       </c>
       <c r="C8" t="n">
-        <v>61.2181206481631</v>
+        <v>35.7149677081741</v>
       </c>
       <c r="D8" t="n">
-        <v>11.5777744052312</v>
+        <v>13.6761871539057</v>
       </c>
       <c r="E8" t="n">
-        <v>151</v>
+        <v>266</v>
       </c>
       <c r="F8" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G8" t="s">
+        <v>3000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>19.3865194734346</v>
+        <v>24.8047047065459</v>
       </c>
       <c r="C9" t="n">
-        <v>23.7636228049237</v>
+        <v>34.1922037910341</v>
       </c>
       <c r="D9" t="n">
-        <v>15.0094161419456</v>
+        <v>15.4172056220576</v>
       </c>
       <c r="E9" t="n">
-        <v>332</v>
+        <v>175</v>
       </c>
       <c r="F9" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G9" t="s">
+        <v>3001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B10" t="n">
-        <v>17.1724986115383</v>
+        <v>36.3979475266971</v>
       </c>
       <c r="C10" t="n">
-        <v>24.4554446207501</v>
+        <v>61.2181206481631</v>
       </c>
       <c r="D10" t="n">
-        <v>9.88955260232654</v>
+        <v>11.5777744052312</v>
       </c>
       <c r="E10" t="n">
-        <v>225</v>
+        <v>151</v>
       </c>
       <c r="F10" t="s">
-        <v>2992</v>
+        <v>2993</v>
+      </c>
+      <c r="G10" t="s">
+        <v>3002</v>
       </c>
     </row>
   </sheetData>
@@ -76576,27 +76636,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>2993</v>
+        <v>3003</v>
       </c>
       <c r="B1" t="s">
-        <v>2994</v>
+        <v>3004</v>
       </c>
       <c r="C1" t="s">
-        <v>2995</v>
+        <v>3005</v>
       </c>
       <c r="D1" t="s">
-        <v>2996</v>
+        <v>3006</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2997</v>
+        <v>3007</v>
       </c>
       <c r="B2" t="s">
-        <v>2998</v>
+        <v>3008</v>
       </c>
       <c r="C2" t="s">
-        <v>2999</v>
+        <v>3009</v>
       </c>
       <c r="D2" t="n">
         <v>2124</v>
@@ -76604,13 +76664,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3000</v>
+        <v>3010</v>
       </c>
       <c r="B3" t="s">
-        <v>3001</v>
+        <v>3011</v>
       </c>
       <c r="C3" t="s">
-        <v>3002</v>
+        <v>3012</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -76618,13 +76678,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3003</v>
+        <v>3013</v>
       </c>
       <c r="B4" t="s">
-        <v>3004</v>
+        <v>3014</v>
       </c>
       <c r="C4" t="s">
-        <v>3005</v>
+        <v>3015</v>
       </c>
       <c r="D4" t="n">
         <v>372</v>
@@ -76632,13 +76692,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3006</v>
+        <v>3016</v>
       </c>
       <c r="B5" t="s">
-        <v>3007</v>
+        <v>3017</v>
       </c>
       <c r="C5" t="s">
-        <v>3005</v>
+        <v>3015</v>
       </c>
       <c r="D5" t="n">
         <v>18</v>
@@ -76646,13 +76706,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3008</v>
+        <v>3018</v>
       </c>
       <c r="B6" t="s">
-        <v>3009</v>
+        <v>3019</v>
       </c>
       <c r="C6" t="s">
-        <v>3010</v>
+        <v>3020</v>
       </c>
       <c r="D6" t="n">
         <v>18</v>
@@ -76660,13 +76720,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>3011</v>
+        <v>3021</v>
       </c>
       <c r="B7" t="s">
-        <v>3012</v>
+        <v>3022</v>
       </c>
       <c r="C7" t="s">
-        <v>3013</v>
+        <v>3023</v>
       </c>
       <c r="D7" t="n">
         <v>1301</v>
@@ -76674,13 +76734,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>3014</v>
+        <v>3024</v>
       </c>
       <c r="B8" t="s">
-        <v>3015</v>
+        <v>3025</v>
       </c>
       <c r="C8" t="s">
-        <v>3016</v>
+        <v>3026</v>
       </c>
       <c r="D8" t="n">
         <v>9</v>

</xml_diff>